<commit_message>
Extend schedule to 5/14 and add deadline pass/fail highlighting
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B4BFaW55DkV287C8tqBYnR
</commit_message>
<xml_diff>
--- a/output/임박재고_소진_시나리오.xlsx
+++ b/output/임박재고_소진_시나리오.xlsx
@@ -735,7 +735,7 @@
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
       <font>
         <b val="1"/>
@@ -745,6 +745,18 @@
         <patternFill patternType="solid">
           <fgColor rgb="00FF0000"/>
           <bgColor rgb="00FF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="0000B050"/>
+          <bgColor rgb="0000B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2446,7 +2458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AD20"/>
+  <dimension ref="A1:AK20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="14.375" bestFit="1" customWidth="1" style="63" min="2" max="2"/>
@@ -2475,8 +2487,16 @@
     <col width="13" customWidth="1" style="63" min="28" max="28"/>
     <col width="13" customWidth="1" style="63" min="29" max="29"/>
     <col width="13" customWidth="1" style="63" min="30" max="30"/>
+    <col width="13" customWidth="1" style="63" min="31" max="31"/>
+    <col width="13" customWidth="1" style="63" min="32" max="32"/>
+    <col width="13" customWidth="1" style="63" min="33" max="33"/>
+    <col width="13" customWidth="1" style="63" min="34" max="34"/>
+    <col width="13" customWidth="1" style="63" min="35" max="35"/>
+    <col width="13" customWidth="1" style="63" min="36" max="36"/>
+    <col width="13" customWidth="1" style="63" min="37" max="37"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="C2" s="0" t="inlineStr">
         <is>
@@ -2590,6 +2610,34 @@
         <f>AC3+7</f>
         <v/>
       </c>
+      <c r="AE3" s="76">
+        <f>AD3+7</f>
+        <v/>
+      </c>
+      <c r="AF3" s="76">
+        <f>AE3+7</f>
+        <v/>
+      </c>
+      <c r="AG3" s="76">
+        <f>AF3+7</f>
+        <v/>
+      </c>
+      <c r="AH3" s="76">
+        <f>AG3+7</f>
+        <v/>
+      </c>
+      <c r="AI3" s="76">
+        <f>AH3+7</f>
+        <v/>
+      </c>
+      <c r="AJ3" s="76">
+        <f>AI3+7</f>
+        <v/>
+      </c>
+      <c r="AK3" s="76">
+        <f>AJ3+7</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -2699,6 +2747,34 @@
       </c>
       <c r="AD4">
         <f>MONTH(AD3)&amp;"월 "&amp;ROUNDUP(DAY(AD3)/7,0)&amp;"주차"</f>
+        <v/>
+      </c>
+      <c r="AE4">
+        <f>MONTH(AE3)&amp;"월 "&amp;ROUNDUP(DAY(AE3)/7,0)&amp;"주차"</f>
+        <v/>
+      </c>
+      <c r="AF4">
+        <f>MONTH(AF3)&amp;"월 "&amp;ROUNDUP(DAY(AF3)/7,0)&amp;"주차"</f>
+        <v/>
+      </c>
+      <c r="AG4">
+        <f>MONTH(AG3)&amp;"월 "&amp;ROUNDUP(DAY(AG3)/7,0)&amp;"주차"</f>
+        <v/>
+      </c>
+      <c r="AH4">
+        <f>MONTH(AH3)&amp;"월 "&amp;ROUNDUP(DAY(AH3)/7,0)&amp;"주차"</f>
+        <v/>
+      </c>
+      <c r="AI4">
+        <f>MONTH(AI3)&amp;"월 "&amp;ROUNDUP(DAY(AI3)/7,0)&amp;"주차"</f>
+        <v/>
+      </c>
+      <c r="AJ4">
+        <f>MONTH(AJ3)&amp;"월 "&amp;ROUNDUP(DAY(AJ3)/7,0)&amp;"주차"</f>
+        <v/>
+      </c>
+      <c r="AK4">
+        <f>MONTH(AK3)&amp;"월 "&amp;ROUNDUP(DAY(AK3)/7,0)&amp;"주차"</f>
         <v/>
       </c>
     </row>
@@ -2822,6 +2898,34 @@
         <f>MIN('데이터 기본'!$G4,MAX(0,SUM('데이터 기본'!$G$4:$G4)-IF($B$5="",$A$5,$B$5)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
+      <c r="AE5" s="80">
+        <f>MIN('데이터 기본'!$G4,MAX(0,SUM('데이터 기본'!$G$4:$G4)-IF($B$5="",$A$5,$B$5)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF5" s="80">
+        <f>MIN('데이터 기본'!$G4,MAX(0,SUM('데이터 기본'!$G$4:$G4)-IF($B$5="",$A$5,$B$5)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG5" s="80">
+        <f>MIN('데이터 기본'!$G4,MAX(0,SUM('데이터 기본'!$G$4:$G4)-IF($B$5="",$A$5,$B$5)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH5" s="80">
+        <f>MIN('데이터 기본'!$G4,MAX(0,SUM('데이터 기본'!$G$4:$G4)-IF($B$5="",$A$5,$B$5)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI5" s="80">
+        <f>MIN('데이터 기본'!$G4,MAX(0,SUM('데이터 기본'!$G$4:$G4)-IF($B$5="",$A$5,$B$5)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ5" s="80">
+        <f>MIN('데이터 기본'!$G4,MAX(0,SUM('데이터 기본'!$G$4:$G4)-IF($B$5="",$A$5,$B$5)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK5" s="80">
+        <f>MIN('데이터 기본'!$G4,MAX(0,SUM('데이터 기본'!$G$4:$G4)-IF($B$5="",$A$5,$B$5)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10">
@@ -2937,6 +3041,34 @@
       </c>
       <c r="AD6" s="83">
         <f>MIN('데이터 기본'!$G5,MAX(0,SUM('데이터 기본'!$G$5:$G5)-IF($B$6="",$A$6,$B$6)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AE6" s="83">
+        <f>MIN('데이터 기본'!$G5,MAX(0,SUM('데이터 기본'!$G$5:$G5)-IF($B$6="",$A$6,$B$6)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF6" s="83">
+        <f>MIN('데이터 기본'!$G5,MAX(0,SUM('데이터 기본'!$G$5:$G5)-IF($B$6="",$A$6,$B$6)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG6" s="83">
+        <f>MIN('데이터 기본'!$G5,MAX(0,SUM('데이터 기본'!$G$5:$G5)-IF($B$6="",$A$6,$B$6)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH6" s="83">
+        <f>MIN('데이터 기본'!$G5,MAX(0,SUM('데이터 기본'!$G$5:$G5)-IF($B$6="",$A$6,$B$6)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI6" s="83">
+        <f>MIN('데이터 기본'!$G5,MAX(0,SUM('데이터 기본'!$G$5:$G5)-IF($B$6="",$A$6,$B$6)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ6" s="83">
+        <f>MIN('데이터 기본'!$G5,MAX(0,SUM('데이터 기본'!$G$5:$G5)-IF($B$6="",$A$6,$B$6)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK6" s="83">
+        <f>MIN('데이터 기본'!$G5,MAX(0,SUM('데이터 기본'!$G$5:$G5)-IF($B$6="",$A$6,$B$6)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
     </row>
@@ -3044,6 +3176,34 @@
         <f>MIN('데이터 기본'!$G6,MAX(0,SUM('데이터 기본'!$G$5:$G6)-IF($B$6="",$A$6,$B$6)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
+      <c r="AE7" s="83">
+        <f>MIN('데이터 기본'!$G6,MAX(0,SUM('데이터 기본'!$G$5:$G6)-IF($B$6="",$A$6,$B$6)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF7" s="83">
+        <f>MIN('데이터 기본'!$G6,MAX(0,SUM('데이터 기본'!$G$5:$G6)-IF($B$6="",$A$6,$B$6)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG7" s="83">
+        <f>MIN('데이터 기본'!$G6,MAX(0,SUM('데이터 기본'!$G$5:$G6)-IF($B$6="",$A$6,$B$6)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH7" s="83">
+        <f>MIN('데이터 기본'!$G6,MAX(0,SUM('데이터 기본'!$G$5:$G6)-IF($B$6="",$A$6,$B$6)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI7" s="83">
+        <f>MIN('데이터 기본'!$G6,MAX(0,SUM('데이터 기본'!$G$5:$G6)-IF($B$6="",$A$6,$B$6)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ7" s="83">
+        <f>MIN('데이터 기본'!$G6,MAX(0,SUM('데이터 기본'!$G$5:$G6)-IF($B$6="",$A$6,$B$6)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK7" s="83">
+        <f>MIN('데이터 기본'!$G6,MAX(0,SUM('데이터 기본'!$G$5:$G6)-IF($B$6="",$A$6,$B$6)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10">
@@ -3161,6 +3321,34 @@
         <f>MIN('데이터 기본'!$G7,MAX(0,SUM('데이터 기본'!$G$7:$G7)-IF($B$8="",$A$8,$B$8)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
+      <c r="AE8" s="83">
+        <f>MIN('데이터 기본'!$G7,MAX(0,SUM('데이터 기본'!$G$7:$G7)-IF($B$8="",$A$8,$B$8)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF8" s="83">
+        <f>MIN('데이터 기본'!$G7,MAX(0,SUM('데이터 기본'!$G$7:$G7)-IF($B$8="",$A$8,$B$8)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG8" s="83">
+        <f>MIN('데이터 기본'!$G7,MAX(0,SUM('데이터 기본'!$G$7:$G7)-IF($B$8="",$A$8,$B$8)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH8" s="83">
+        <f>MIN('데이터 기본'!$G7,MAX(0,SUM('데이터 기본'!$G$7:$G7)-IF($B$8="",$A$8,$B$8)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI8" s="83">
+        <f>MIN('데이터 기본'!$G7,MAX(0,SUM('데이터 기본'!$G$7:$G7)-IF($B$8="",$A$8,$B$8)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ8" s="83">
+        <f>MIN('데이터 기본'!$G7,MAX(0,SUM('데이터 기본'!$G$7:$G7)-IF($B$8="",$A$8,$B$8)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK8" s="83">
+        <f>MIN('데이터 기본'!$G7,MAX(0,SUM('데이터 기본'!$G$7:$G7)-IF($B$8="",$A$8,$B$8)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="10">
@@ -3280,6 +3468,34 @@
       </c>
       <c r="AD9" s="83">
         <f>MIN('데이터 기본'!$G8,MAX(0,SUM('데이터 기본'!$G$8:$G8)-IF($B$9="",$A$9,$B$9)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AE9" s="83">
+        <f>MIN('데이터 기본'!$G8,MAX(0,SUM('데이터 기본'!$G$8:$G8)-IF($B$9="",$A$9,$B$9)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF9" s="83">
+        <f>MIN('데이터 기본'!$G8,MAX(0,SUM('데이터 기본'!$G$8:$G8)-IF($B$9="",$A$9,$B$9)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG9" s="83">
+        <f>MIN('데이터 기본'!$G8,MAX(0,SUM('데이터 기본'!$G$8:$G8)-IF($B$9="",$A$9,$B$9)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH9" s="83">
+        <f>MIN('데이터 기본'!$G8,MAX(0,SUM('데이터 기본'!$G$8:$G8)-IF($B$9="",$A$9,$B$9)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI9" s="83">
+        <f>MIN('데이터 기본'!$G8,MAX(0,SUM('데이터 기본'!$G$8:$G8)-IF($B$9="",$A$9,$B$9)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ9" s="83">
+        <f>MIN('데이터 기본'!$G8,MAX(0,SUM('데이터 기본'!$G$8:$G8)-IF($B$9="",$A$9,$B$9)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK9" s="83">
+        <f>MIN('데이터 기본'!$G8,MAX(0,SUM('데이터 기본'!$G$8:$G8)-IF($B$9="",$A$9,$B$9)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
     </row>
@@ -3387,6 +3603,34 @@
         <f>MIN('데이터 기본'!$G9,MAX(0,SUM('데이터 기본'!$G$8:$G9)-IF($B$9="",$A$9,$B$9)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
+      <c r="AE10" s="83">
+        <f>MIN('데이터 기본'!$G9,MAX(0,SUM('데이터 기본'!$G$8:$G9)-IF($B$9="",$A$9,$B$9)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF10" s="83">
+        <f>MIN('데이터 기본'!$G9,MAX(0,SUM('데이터 기본'!$G$8:$G9)-IF($B$9="",$A$9,$B$9)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG10" s="83">
+        <f>MIN('데이터 기본'!$G9,MAX(0,SUM('데이터 기본'!$G$8:$G9)-IF($B$9="",$A$9,$B$9)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH10" s="83">
+        <f>MIN('데이터 기본'!$G9,MAX(0,SUM('데이터 기본'!$G$8:$G9)-IF($B$9="",$A$9,$B$9)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI10" s="83">
+        <f>MIN('데이터 기본'!$G9,MAX(0,SUM('데이터 기본'!$G$8:$G9)-IF($B$9="",$A$9,$B$9)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ10" s="83">
+        <f>MIN('데이터 기본'!$G9,MAX(0,SUM('데이터 기본'!$G$8:$G9)-IF($B$9="",$A$9,$B$9)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK10" s="83">
+        <f>MIN('데이터 기본'!$G9,MAX(0,SUM('데이터 기본'!$G$8:$G9)-IF($B$9="",$A$9,$B$9)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="72" t="n"/>
@@ -3492,6 +3736,34 @@
         <f>MIN('데이터 기본'!$G10,MAX(0,SUM('데이터 기본'!$G$8:$G10)-IF($B$9="",$A$9,$B$9)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
+      <c r="AE11" s="83">
+        <f>MIN('데이터 기본'!$G10,MAX(0,SUM('데이터 기본'!$G$8:$G10)-IF($B$9="",$A$9,$B$9)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF11" s="83">
+        <f>MIN('데이터 기본'!$G10,MAX(0,SUM('데이터 기본'!$G$8:$G10)-IF($B$9="",$A$9,$B$9)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG11" s="83">
+        <f>MIN('데이터 기본'!$G10,MAX(0,SUM('데이터 기본'!$G$8:$G10)-IF($B$9="",$A$9,$B$9)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH11" s="83">
+        <f>MIN('데이터 기본'!$G10,MAX(0,SUM('데이터 기본'!$G$8:$G10)-IF($B$9="",$A$9,$B$9)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI11" s="83">
+        <f>MIN('데이터 기본'!$G10,MAX(0,SUM('데이터 기본'!$G$8:$G10)-IF($B$9="",$A$9,$B$9)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ11" s="83">
+        <f>MIN('데이터 기본'!$G10,MAX(0,SUM('데이터 기본'!$G$8:$G10)-IF($B$9="",$A$9,$B$9)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK11" s="83">
+        <f>MIN('데이터 기본'!$G10,MAX(0,SUM('데이터 기본'!$G$8:$G10)-IF($B$9="",$A$9,$B$9)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="71" t="n"/>
@@ -3597,6 +3869,34 @@
         <f>MIN('데이터 기본'!$G11,MAX(0,SUM('데이터 기본'!$G$8:$G11)-IF($B$9="",$A$9,$B$9)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
+      <c r="AE12" s="83">
+        <f>MIN('데이터 기본'!$G11,MAX(0,SUM('데이터 기본'!$G$8:$G11)-IF($B$9="",$A$9,$B$9)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF12" s="83">
+        <f>MIN('데이터 기본'!$G11,MAX(0,SUM('데이터 기본'!$G$8:$G11)-IF($B$9="",$A$9,$B$9)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG12" s="83">
+        <f>MIN('데이터 기본'!$G11,MAX(0,SUM('데이터 기본'!$G$8:$G11)-IF($B$9="",$A$9,$B$9)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH12" s="83">
+        <f>MIN('데이터 기본'!$G11,MAX(0,SUM('데이터 기본'!$G$8:$G11)-IF($B$9="",$A$9,$B$9)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI12" s="83">
+        <f>MIN('데이터 기본'!$G11,MAX(0,SUM('데이터 기본'!$G$8:$G11)-IF($B$9="",$A$9,$B$9)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ12" s="83">
+        <f>MIN('데이터 기본'!$G11,MAX(0,SUM('데이터 기본'!$G$8:$G11)-IF($B$9="",$A$9,$B$9)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK12" s="83">
+        <f>MIN('데이터 기본'!$G11,MAX(0,SUM('데이터 기본'!$G$8:$G11)-IF($B$9="",$A$9,$B$9)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10">
@@ -3712,6 +4012,34 @@
       </c>
       <c r="AD13" s="83">
         <f>MIN('데이터 기본'!$G12,MAX(0,SUM('데이터 기본'!$G$12:$G12)-IF($B$13="",$A$13,$B$13)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AE13" s="83">
+        <f>MIN('데이터 기본'!$G12,MAX(0,SUM('데이터 기본'!$G$12:$G12)-IF($B$13="",$A$13,$B$13)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF13" s="83">
+        <f>MIN('데이터 기본'!$G12,MAX(0,SUM('데이터 기본'!$G$12:$G12)-IF($B$13="",$A$13,$B$13)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG13" s="83">
+        <f>MIN('데이터 기본'!$G12,MAX(0,SUM('데이터 기본'!$G$12:$G12)-IF($B$13="",$A$13,$B$13)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH13" s="83">
+        <f>MIN('데이터 기본'!$G12,MAX(0,SUM('데이터 기본'!$G$12:$G12)-IF($B$13="",$A$13,$B$13)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI13" s="83">
+        <f>MIN('데이터 기본'!$G12,MAX(0,SUM('데이터 기본'!$G$12:$G12)-IF($B$13="",$A$13,$B$13)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ13" s="83">
+        <f>MIN('데이터 기본'!$G12,MAX(0,SUM('데이터 기본'!$G$12:$G12)-IF($B$13="",$A$13,$B$13)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK13" s="83">
+        <f>MIN('데이터 기본'!$G12,MAX(0,SUM('데이터 기본'!$G$12:$G12)-IF($B$13="",$A$13,$B$13)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
     </row>
@@ -3819,6 +4147,34 @@
         <f>MIN('데이터 기본'!$G13,MAX(0,SUM('데이터 기본'!$G$12:$G13)-IF($B$13="",$A$13,$B$13)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
+      <c r="AE14" s="83">
+        <f>MIN('데이터 기본'!$G13,MAX(0,SUM('데이터 기본'!$G$12:$G13)-IF($B$13="",$A$13,$B$13)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF14" s="83">
+        <f>MIN('데이터 기본'!$G13,MAX(0,SUM('데이터 기본'!$G$12:$G13)-IF($B$13="",$A$13,$B$13)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG14" s="83">
+        <f>MIN('데이터 기본'!$G13,MAX(0,SUM('데이터 기본'!$G$12:$G13)-IF($B$13="",$A$13,$B$13)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH14" s="83">
+        <f>MIN('데이터 기본'!$G13,MAX(0,SUM('데이터 기본'!$G$12:$G13)-IF($B$13="",$A$13,$B$13)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI14" s="83">
+        <f>MIN('데이터 기본'!$G13,MAX(0,SUM('데이터 기본'!$G$12:$G13)-IF($B$13="",$A$13,$B$13)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ14" s="83">
+        <f>MIN('데이터 기본'!$G13,MAX(0,SUM('데이터 기본'!$G$12:$G13)-IF($B$13="",$A$13,$B$13)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK14" s="83">
+        <f>MIN('데이터 기본'!$G13,MAX(0,SUM('데이터 기본'!$G$12:$G13)-IF($B$13="",$A$13,$B$13)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="72" t="n"/>
@@ -3924,6 +4280,34 @@
         <f>MIN('데이터 기본'!$G14,MAX(0,SUM('데이터 기본'!$G$12:$G14)-IF($B$13="",$A$13,$B$13)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
+      <c r="AE15" s="83">
+        <f>MIN('데이터 기본'!$G14,MAX(0,SUM('데이터 기본'!$G$12:$G14)-IF($B$13="",$A$13,$B$13)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF15" s="83">
+        <f>MIN('데이터 기본'!$G14,MAX(0,SUM('데이터 기본'!$G$12:$G14)-IF($B$13="",$A$13,$B$13)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG15" s="83">
+        <f>MIN('데이터 기본'!$G14,MAX(0,SUM('데이터 기본'!$G$12:$G14)-IF($B$13="",$A$13,$B$13)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH15" s="83">
+        <f>MIN('데이터 기본'!$G14,MAX(0,SUM('데이터 기본'!$G$12:$G14)-IF($B$13="",$A$13,$B$13)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI15" s="83">
+        <f>MIN('데이터 기본'!$G14,MAX(0,SUM('데이터 기본'!$G$12:$G14)-IF($B$13="",$A$13,$B$13)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ15" s="83">
+        <f>MIN('데이터 기본'!$G14,MAX(0,SUM('데이터 기본'!$G$12:$G14)-IF($B$13="",$A$13,$B$13)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK15" s="83">
+        <f>MIN('데이터 기본'!$G14,MAX(0,SUM('데이터 기본'!$G$12:$G14)-IF($B$13="",$A$13,$B$13)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="71" t="n"/>
@@ -4029,6 +4413,34 @@
         <f>MIN('데이터 기본'!$G15,MAX(0,SUM('데이터 기본'!$G$12:$G15)-IF($B$13="",$A$13,$B$13)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
+      <c r="AE16" s="83">
+        <f>MIN('데이터 기본'!$G15,MAX(0,SUM('데이터 기본'!$G$12:$G15)-IF($B$13="",$A$13,$B$13)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF16" s="83">
+        <f>MIN('데이터 기본'!$G15,MAX(0,SUM('데이터 기본'!$G$12:$G15)-IF($B$13="",$A$13,$B$13)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG16" s="83">
+        <f>MIN('데이터 기본'!$G15,MAX(0,SUM('데이터 기본'!$G$12:$G15)-IF($B$13="",$A$13,$B$13)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH16" s="83">
+        <f>MIN('데이터 기본'!$G15,MAX(0,SUM('데이터 기본'!$G$12:$G15)-IF($B$13="",$A$13,$B$13)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI16" s="83">
+        <f>MIN('데이터 기본'!$G15,MAX(0,SUM('데이터 기본'!$G$12:$G15)-IF($B$13="",$A$13,$B$13)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ16" s="83">
+        <f>MIN('데이터 기본'!$G15,MAX(0,SUM('데이터 기본'!$G$12:$G15)-IF($B$13="",$A$13,$B$13)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK16" s="83">
+        <f>MIN('데이터 기본'!$G15,MAX(0,SUM('데이터 기본'!$G$12:$G15)-IF($B$13="",$A$13,$B$13)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="10">
@@ -4148,6 +4560,34 @@
       </c>
       <c r="AD17" s="83">
         <f>MIN('데이터 기본'!$G16,MAX(0,SUM('데이터 기본'!$G$16:$G16)-IF($B$17="",$A$17,$B$17)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AE17" s="83">
+        <f>MIN('데이터 기본'!$G16,MAX(0,SUM('데이터 기본'!$G$16:$G16)-IF($B$17="",$A$17,$B$17)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF17" s="83">
+        <f>MIN('데이터 기본'!$G16,MAX(0,SUM('데이터 기본'!$G$16:$G16)-IF($B$17="",$A$17,$B$17)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG17" s="83">
+        <f>MIN('데이터 기본'!$G16,MAX(0,SUM('데이터 기본'!$G$16:$G16)-IF($B$17="",$A$17,$B$17)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH17" s="83">
+        <f>MIN('데이터 기본'!$G16,MAX(0,SUM('데이터 기본'!$G$16:$G16)-IF($B$17="",$A$17,$B$17)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI17" s="83">
+        <f>MIN('데이터 기본'!$G16,MAX(0,SUM('데이터 기본'!$G$16:$G16)-IF($B$17="",$A$17,$B$17)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ17" s="83">
+        <f>MIN('데이터 기본'!$G16,MAX(0,SUM('데이터 기본'!$G$16:$G16)-IF($B$17="",$A$17,$B$17)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK17" s="83">
+        <f>MIN('데이터 기본'!$G16,MAX(0,SUM('데이터 기본'!$G$16:$G16)-IF($B$17="",$A$17,$B$17)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
     </row>
@@ -4255,6 +4695,34 @@
         <f>MIN('데이터 기본'!$G17,MAX(0,SUM('데이터 기본'!$G$16:$G17)-IF($B$17="",$A$17,$B$17)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
+      <c r="AE18" s="83">
+        <f>MIN('데이터 기본'!$G17,MAX(0,SUM('데이터 기본'!$G$16:$G17)-IF($B$17="",$A$17,$B$17)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF18" s="83">
+        <f>MIN('데이터 기본'!$G17,MAX(0,SUM('데이터 기본'!$G$16:$G17)-IF($B$17="",$A$17,$B$17)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG18" s="83">
+        <f>MIN('데이터 기본'!$G17,MAX(0,SUM('데이터 기본'!$G$16:$G17)-IF($B$17="",$A$17,$B$17)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH18" s="83">
+        <f>MIN('데이터 기본'!$G17,MAX(0,SUM('데이터 기본'!$G$16:$G17)-IF($B$17="",$A$17,$B$17)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI18" s="83">
+        <f>MIN('데이터 기본'!$G17,MAX(0,SUM('데이터 기본'!$G$16:$G17)-IF($B$17="",$A$17,$B$17)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ18" s="83">
+        <f>MIN('데이터 기본'!$G17,MAX(0,SUM('데이터 기본'!$G$16:$G17)-IF($B$17="",$A$17,$B$17)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK18" s="83">
+        <f>MIN('데이터 기본'!$G17,MAX(0,SUM('데이터 기본'!$G$16:$G17)-IF($B$17="",$A$17,$B$17)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="73">
@@ -4370,6 +4838,34 @@
       </c>
       <c r="AD19" s="83">
         <f>MIN('데이터 기본'!$G18,MAX(0,SUM('데이터 기본'!$G$18:$G18)-IF($B$19="",$A$19,$B$19)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AE19" s="83">
+        <f>MIN('데이터 기본'!$G18,MAX(0,SUM('데이터 기본'!$G$18:$G18)-IF($B$19="",$A$19,$B$19)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF19" s="83">
+        <f>MIN('데이터 기본'!$G18,MAX(0,SUM('데이터 기본'!$G$18:$G18)-IF($B$19="",$A$19,$B$19)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG19" s="83">
+        <f>MIN('데이터 기본'!$G18,MAX(0,SUM('데이터 기본'!$G$18:$G18)-IF($B$19="",$A$19,$B$19)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH19" s="83">
+        <f>MIN('데이터 기본'!$G18,MAX(0,SUM('데이터 기본'!$G$18:$G18)-IF($B$19="",$A$19,$B$19)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI19" s="83">
+        <f>MIN('데이터 기본'!$G18,MAX(0,SUM('데이터 기본'!$G$18:$G18)-IF($B$19="",$A$19,$B$19)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ19" s="83">
+        <f>MIN('데이터 기본'!$G18,MAX(0,SUM('데이터 기본'!$G$18:$G18)-IF($B$19="",$A$19,$B$19)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK19" s="83">
+        <f>MIN('데이터 기본'!$G18,MAX(0,SUM('데이터 기본'!$G$18:$G18)-IF($B$19="",$A$19,$B$19)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
     </row>
@@ -4475,6 +4971,34 @@
       </c>
       <c r="AD20" s="86">
         <f>MIN('데이터 기본'!$G19,MAX(0,SUM('데이터 기본'!$G$18:$G19)-IF($B$19="",$A$19,$B$19)*MAX(0,AD$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AE20" s="86">
+        <f>MIN('데이터 기본'!$G19,MAX(0,SUM('데이터 기본'!$G$18:$G19)-IF($B$19="",$A$19,$B$19)*MAX(0,AE$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AF20" s="86">
+        <f>MIN('데이터 기본'!$G19,MAX(0,SUM('데이터 기본'!$G$18:$G19)-IF($B$19="",$A$19,$B$19)*MAX(0,AF$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AG20" s="86">
+        <f>MIN('데이터 기본'!$G19,MAX(0,SUM('데이터 기본'!$G$18:$G19)-IF($B$19="",$A$19,$B$19)*MAX(0,AG$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AH20" s="86">
+        <f>MIN('데이터 기본'!$G19,MAX(0,SUM('데이터 기본'!$G$18:$G19)-IF($B$19="",$A$19,$B$19)*MAX(0,AH$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AI20" s="86">
+        <f>MIN('데이터 기본'!$G19,MAX(0,SUM('데이터 기본'!$G$18:$G19)-IF($B$19="",$A$19,$B$19)*MAX(0,AI$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AJ20" s="86">
+        <f>MIN('데이터 기본'!$G19,MAX(0,SUM('데이터 기본'!$G$18:$G19)-IF($B$19="",$A$19,$B$19)*MAX(0,AJ$3-'데이터 기본'!$B$1)))</f>
+        <v/>
+      </c>
+      <c r="AK20" s="86">
+        <f>MIN('데이터 기본'!$G19,MAX(0,SUM('데이터 기본'!$G$18:$G19)-IF($B$19="",$A$19,$B$19)*MAX(0,AK$3-'데이터 기본'!$B$1)))</f>
         <v/>
       </c>
     </row>
@@ -4504,9 +5028,212 @@
     <mergeCell ref="A9:A12"/>
     <mergeCell ref="D6:D7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:AD20">
+  <conditionalFormatting sqref="G5:AK5">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND(G5&lt;=0,ISNUMBER(F5),F5&gt;0)</formula>
+      <formula>AND(AND(ISNUMBER($B$5),$B$5&gt;0),G5&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F5">
+    <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$5),$B$5&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$4:$G4)/$B$5&lt;=$F5-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>AND(ISNUMBER($B$5),$B$5&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G6:AK6">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$6),$B$6&gt;0),G6&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F6">
+    <cfRule type="expression" priority="5" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$6),$B$6&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$5:$G5)/$B$6&lt;=$F6-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="0">
+      <formula>AND(ISNUMBER($B$6),$B$6&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7:AK7">
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$6),$B$6&gt;0),G7&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F7">
+    <cfRule type="expression" priority="8" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$6),$B$6&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$5:$G6)/$B$6&lt;=$F7-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="0">
+      <formula>AND(ISNUMBER($B$6),$B$6&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8:AK8">
+    <cfRule type="expression" priority="10" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$8),$B$8&gt;0),G8&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F8">
+    <cfRule type="expression" priority="11" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$8),$B$8&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$7:$G7)/$B$8&lt;=$F8-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="0">
+      <formula>AND(ISNUMBER($B$8),$B$8&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9:AK9">
+    <cfRule type="expression" priority="13" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$9),$B$9&gt;0),G9&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F9">
+    <cfRule type="expression" priority="14" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$9),$B$9&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$8:$G8)/$B$9&lt;=$F9-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="0">
+      <formula>AND(ISNUMBER($B$9),$B$9&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G10:AK10">
+    <cfRule type="expression" priority="16" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$9),$B$9&gt;0),G10&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F10">
+    <cfRule type="expression" priority="17" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$9),$B$9&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$8:$G9)/$B$9&lt;=$F10-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="0">
+      <formula>AND(ISNUMBER($B$9),$B$9&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11:AK11">
+    <cfRule type="expression" priority="19" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$9),$B$9&gt;0),G11&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F11">
+    <cfRule type="expression" priority="20" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$9),$B$9&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$8:$G10)/$B$9&lt;=$F11-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="21" dxfId="0">
+      <formula>AND(ISNUMBER($B$9),$B$9&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G12:AK12">
+    <cfRule type="expression" priority="22" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$9),$B$9&gt;0),G12&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F12">
+    <cfRule type="expression" priority="23" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$9),$B$9&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$8:$G11)/$B$9&lt;=$F12-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="24" dxfId="0">
+      <formula>AND(ISNUMBER($B$9),$B$9&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G13:AK13">
+    <cfRule type="expression" priority="25" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$13),$B$13&gt;0),G13&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F13">
+    <cfRule type="expression" priority="26" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$13),$B$13&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$12:$G12)/$B$13&lt;=$F13-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="27" dxfId="0">
+      <formula>AND(ISNUMBER($B$13),$B$13&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G14:AK14">
+    <cfRule type="expression" priority="28" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$13),$B$13&gt;0),G14&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F14">
+    <cfRule type="expression" priority="29" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$13),$B$13&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$12:$G13)/$B$13&lt;=$F14-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="30" dxfId="0">
+      <formula>AND(ISNUMBER($B$13),$B$13&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G15:AK15">
+    <cfRule type="expression" priority="31" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$13),$B$13&gt;0),G15&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F15">
+    <cfRule type="expression" priority="32" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$13),$B$13&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$12:$G14)/$B$13&lt;=$F15-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="33" dxfId="0">
+      <formula>AND(ISNUMBER($B$13),$B$13&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16:AK16">
+    <cfRule type="expression" priority="34" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$13),$B$13&gt;0),G16&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F16">
+    <cfRule type="expression" priority="35" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$13),$B$13&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$12:$G15)/$B$13&lt;=$F16-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="36" dxfId="0">
+      <formula>AND(ISNUMBER($B$13),$B$13&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17:AK17">
+    <cfRule type="expression" priority="37" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$17),$B$17&gt;0),G17&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F17">
+    <cfRule type="expression" priority="38" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$17),$B$17&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$16:$G16)/$B$17&lt;=$F17-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="39" dxfId="0">
+      <formula>AND(ISNUMBER($B$17),$B$17&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G18:AK18">
+    <cfRule type="expression" priority="40" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$17),$B$17&gt;0),G18&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F18">
+    <cfRule type="expression" priority="41" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$17),$B$17&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$16:$G17)/$B$17&lt;=$F18-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="42" dxfId="0">
+      <formula>AND(ISNUMBER($B$17),$B$17&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19:AK19">
+    <cfRule type="expression" priority="43" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$19),$B$19&gt;0),G19&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F19">
+    <cfRule type="expression" priority="44" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$19),$B$19&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$18:$G18)/$B$19&lt;=$F19-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="45" dxfId="0">
+      <formula>AND(ISNUMBER($B$19),$B$19&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G20:AK20">
+    <cfRule type="expression" priority="46" dxfId="0">
+      <formula>AND(AND(ISNUMBER($B$19),$B$19&gt;0),G20&lt;=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F20">
+    <cfRule type="expression" priority="47" dxfId="1" stopIfTrue="1">
+      <formula>AND(AND(ISNUMBER($B$19),$B$19&gt;0),'데이터 기본'!$B$1+SUM('데이터 기본'!$G$18:$G19)/$B$19&lt;=$F20-30)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="48" dxfId="0">
+      <formula>AND(ISNUMBER($B$19),$B$19&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>